<commit_message>
Update frontier forecasts and responsive explorer
</commit_message>
<xml_diff>
--- a/outputs/019f6c42-2d53-7743-ab07-6293e2618dd7/frontier_parameter_chronological_backtest_2026-07-17.xlsx
+++ b/outputs/019f6c42-2d53-7743-ab07-6293e2618dd7/frontier_parameter_chronological_backtest_2026-07-17.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Executive Summary" sheetId="1" r:id="R32f6f6ff948c4580"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Model Comparison" sheetId="2" r:id="R3fd6ad1e087648a1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="OOS Predictions" sheetId="3" r:id="Rfad94430f52b47df"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ensemble Backtest" sheetId="4" r:id="R0885d4726e06478c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="External Checks" sheetId="5" r:id="R38488a1891a24c71"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Method and Limits" sheetId="6" r:id="Rdfc0229453634c33"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Executive Summary" sheetId="1" r:id="R900a208d28e54866"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Model Comparison" sheetId="2" r:id="Rc01474a683be45bf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="OOS Predictions" sheetId="3" r:id="R4a3b241c498d4b7b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ensemble Backtest" sheetId="4" r:id="R8aeaa0af46d64873"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="External Checks" sheetId="5" r:id="R9d824568e450481f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Method and Limits" sheetId="6" r:id="R5c81c91884c04ab0"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -15,7 +15,7 @@
 <file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
 <x:comments xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:authors>
-    <x:author>tc={74F4DC58-EA34-4D12-3A93-964F6E42178B}</x:author>
+    <x:author>tc={5BCCBB34-6BD6-50D0-FA5E-E54C284F0A05}</x:author>
   </x:authors>
   <x:commentList>
     <x:comment ref="C12" authorId="0">
@@ -35,8 +35,8 @@
 <file path=xl/comments2.xml><?xml version="1.0" encoding="utf-8"?>
 <x:comments xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:authors>
-    <x:author>tc={3FA342DA-22D3-604E-DA3C-FFC532DEF03E}</x:author>
-    <x:author>tc={C90D3448-B695-AB30-08D3-3FC90653F39F}</x:author>
+    <x:author>tc={ED4B7BBB-4E4D-83D4-B96A-549733F9ED0A}</x:author>
+    <x:author>tc={109F75FB-593F-AE95-3E31-EAD36EBA5B97}</x:author>
   </x:authors>
   <x:commentList>
     <x:comment ref="B26" authorId="0">
@@ -588,7 +588,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R2aa6b9a3e1fb4222"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R40cf17a9c1d74af3"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -599,7 +599,7 @@
 
 <file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
 <xltc:personList xmlns:xltc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments">
-  <xltc:person displayName="Codex" id="{FA841AD2-A7F4-41B1-9968-3B84A468A72B}"/>
+  <xltc:person displayName="Codex" id="{9880DB29-1A54-415F-8236-4210258137F2}"/>
 </xltc:personList>
 </file>
 
@@ -873,7 +873,7 @@
 
 <file path=xl/threadedcomments/threadedcomment.xml><?xml version="1.0" encoding="utf-8"?>
 <xltc:ThreadedComments xmlns:xltc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments">
-  <xltc:threadedComment ref="C12" dT="2026-08-01T16:01:45.642" personId="{FA841AD2-A7F4-41B1-9968-3B84A468A72B}" id="{74F4DC58-EA34-4D12-3A93-964F6E42178B}">
+  <xltc:threadedComment ref="C12" dT="2026-08-01T18:06:22.458" personId="{9880DB29-1A54-415F-8236-4210258137F2}" id="{5BCCBB34-6BD6-50D0-FA5E-E54C284F0A05}">
     <xltc:text>The ensemble row is not a full-pipeline backtest: price and crowd are unavailable, and models contribute only where at least two component OOS predictions match conservatively.</xltc:text>
   </xltc:threadedComment>
 </xltc:ThreadedComments>
@@ -881,10 +881,10 @@
 
 <file path=xl/threadedcomments/threadedcomment2.xml><?xml version="1.0" encoding="utf-8"?>
 <xltc:ThreadedComments xmlns:xltc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments">
-  <xltc:threadedComment ref="B26" dT="2026-08-01T16:01:45.644" personId="{FA841AD2-A7F4-41B1-9968-3B84A468A72B}" id="{3FA342DA-22D3-604E-DA3C-FFC532DEF03E}">
+  <xltc:threadedComment ref="B26" dT="2026-08-01T18:06:22.458" personId="{9880DB29-1A54-415F-8236-4210258137F2}" id="{ED4B7BBB-4E4D-83D4-B96A-549733F9ED0A}">
     <xltc:text>The ECI live branch is a 60/40 score-only/dated log blend. The date coefficient remains because chronology matters, but the backtest does not support treating it as a stable law.</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="B27" dT="2026-08-01T16:01:45.644" personId="{FA841AD2-A7F4-41B1-9968-3B84A468A72B}" id="{C90D3448-B695-AB30-08D3-3FC90653F39F}">
+  <xltc:threadedComment ref="B27" dT="2026-08-01T18:06:22.458" personId="{9880DB29-1A54-415F-8236-4210258137F2}" id="{109F75FB-593F-AE95-3E31-EAD36EBA5B97}">
     <xltc:text>No-CoT retains the user's 50% evidence-level prior in the live model. This backtest shows useful signal but does not identify that weight as optimal.</xltc:text>
   </xltc:threadedComment>
 </xltc:ThreadedComments>
@@ -1454,8 +1454,8 @@
     </x:cfRule>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf9e96a0d5a494a5b"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ree41f3d7be1b4b22"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd784a177074f4914"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb9d9ac4a54d24366"/>
 </x:worksheet>
 </file>
 
@@ -3257,7 +3257,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd59bc331f9ed4907"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8a0afd6a24bd4c66"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -19811,7 +19811,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R003a4e82b9b24275"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4758edda1305431a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -21527,7 +21527,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R03ea9eec0d444b4f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8ce8dbed486d4b5a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -21789,7 +21789,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R881778dd71784309"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R05ac6106ab8e418f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -22723,6 +22723,6 @@
     <x:cfRule type="containsText" dxfId="4" priority="1" operator="containsText" text="High"/>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2a61b0b6c07a419f"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2c32aab4b1a44b0d"/>
 </x:worksheet>
 </file>
</xml_diff>